<commit_message>
feat: land race token equipment D-080 with Q21-Q27 grave prefabs
Add human/elf/orc token configs, Dig HUD GM grant/spend, grave quality coverage, and SPEC closeout for spawn-weight bonuses.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Gravedigger2026/Assets/ConfigTables/Mode2/Excel/主角_装备配置表_Protagonist_ProtagonistEquipmentConfig.xlsx
+++ b/Gravedigger2026/Assets/ConfigTables/Mode2/Excel/主角_装备配置表_Protagonist_ProtagonistEquipmentConfig.xlsx
@@ -16,14 +16,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="21">
-    <font>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <color theme="1"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
+  <fonts count="20">
     <font>
       <name val="宋体"/>
       <charset val="134"/>
@@ -176,7 +169,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="34">
+  <fills count="35">
     <fill>
       <patternFill/>
     </fill>
@@ -186,6 +179,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.8"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -484,165 +483,168 @@
     </border>
   </borders>
   <cellStyleXfs count="49">
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="4" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="5" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="4" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="6" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="4" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="5" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="4" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="6" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="9" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="10" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="11" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="14" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="15" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="18" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="19" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="22" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="23" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="26" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="27" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="30" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="31" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="33" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="18" fillId="34" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -1056,12 +1058,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I33"/>
+  <dimension ref="A1:J43"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
-    <col width="22.625" customWidth="1" style="5" min="1" max="1"/>
-    <col width="16.875" customWidth="1" style="5" min="4" max="4"/>
-    <col width="33.875" customWidth="1" style="5" min="8" max="8"/>
+    <col width="22.625" customWidth="1" style="4" min="1" max="1"/>
+    <col width="16.875" customWidth="1" style="4" min="4" max="4"/>
+    <col width="33.875" customWidth="1" style="4" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1231,7 +1233,7 @@
           <t>1</t>
         </is>
       </c>
-      <c r="F4" s="6" t="inlineStr">
+      <c r="F4" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -1241,7 +1243,7 @@
           <t>Dig</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>DigCursorRadius_0.06</t>
         </is>
@@ -1278,7 +1280,7 @@
           <t>1</t>
         </is>
       </c>
-      <c r="F5" s="6" t="n">
+      <c r="F5" s="5" t="n">
         <v>2</v>
       </c>
       <c r="G5" t="inlineStr">
@@ -1286,7 +1288,7 @@
           <t>Dig</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>DigCursorRadius_0.16</t>
         </is>
@@ -1323,7 +1325,7 @@
           <t>1</t>
         </is>
       </c>
-      <c r="F6" s="6" t="n">
+      <c r="F6" s="5" t="n">
         <v>3</v>
       </c>
       <c r="G6" t="inlineStr">
@@ -1331,7 +1333,7 @@
           <t>Dig</t>
         </is>
       </c>
-      <c r="H6" s="3" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>DigCursorRadius_0.26</t>
         </is>
@@ -1368,7 +1370,7 @@
           <t>1</t>
         </is>
       </c>
-      <c r="F7" s="6" t="n">
+      <c r="F7" s="5" t="n">
         <v>4</v>
       </c>
       <c r="G7" t="inlineStr">
@@ -1376,7 +1378,7 @@
           <t>Dig</t>
         </is>
       </c>
-      <c r="H7" s="3" t="inlineStr">
+      <c r="H7" t="inlineStr">
         <is>
           <t>DigCursorRadius_0.36</t>
         </is>
@@ -1408,7 +1410,7 @@
           <t>Icon_IronShovel</t>
         </is>
       </c>
-      <c r="F8" s="6" t="n">
+      <c r="F8" s="5" t="n">
         <v>5</v>
       </c>
       <c r="G8" t="inlineStr">
@@ -1416,7 +1418,7 @@
           <t>Dig</t>
         </is>
       </c>
-      <c r="H8" s="3" t="inlineStr">
+      <c r="H8" t="inlineStr">
         <is>
           <t>DigCursorRadius_0.46</t>
         </is>
@@ -1453,7 +1455,7 @@
           <t>1</t>
         </is>
       </c>
-      <c r="F9" s="6" t="inlineStr">
+      <c r="F9" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -1463,7 +1465,7 @@
           <t>Dig</t>
         </is>
       </c>
-      <c r="H9" s="3" t="inlineStr">
+      <c r="H9" t="inlineStr">
         <is>
           <t>GraveSpawnWeightBonus_Q4_10|GraveSpawnWeightBonus_Q5_10|GraveSpawnWeightBonus_Q6_10</t>
         </is>
@@ -1500,7 +1502,7 @@
           <t>1</t>
         </is>
       </c>
-      <c r="F10" s="6" t="n">
+      <c r="F10" s="5" t="n">
         <v>2</v>
       </c>
       <c r="G10" t="inlineStr">
@@ -1508,7 +1510,7 @@
           <t>Dig</t>
         </is>
       </c>
-      <c r="H10" s="3" t="inlineStr">
+      <c r="H10" t="inlineStr">
         <is>
           <t>GraveSpawnWeightBonus_Q4_20|GraveSpawnWeightBonus_Q5_20|GraveSpawnWeightBonus_Q6_20</t>
         </is>
@@ -1545,7 +1547,7 @@
           <t>1</t>
         </is>
       </c>
-      <c r="F11" s="6" t="n">
+      <c r="F11" s="5" t="n">
         <v>3</v>
       </c>
       <c r="G11" t="inlineStr">
@@ -1553,7 +1555,7 @@
           <t>Dig</t>
         </is>
       </c>
-      <c r="H11" s="3" t="inlineStr">
+      <c r="H11" t="inlineStr">
         <is>
           <t>GraveSpawnWeightBonus_Q4_30|GraveSpawnWeightBonus_Q5_30|GraveSpawnWeightBonus_Q6_30</t>
         </is>
@@ -1590,7 +1592,7 @@
           <t>1</t>
         </is>
       </c>
-      <c r="F12" s="6" t="n">
+      <c r="F12" s="5" t="n">
         <v>4</v>
       </c>
       <c r="G12" t="inlineStr">
@@ -1598,7 +1600,7 @@
           <t>Dig</t>
         </is>
       </c>
-      <c r="H12" s="3" t="inlineStr">
+      <c r="H12" t="inlineStr">
         <is>
           <t>GraveSpawnWeightBonus_Q4_40|GraveSpawnWeightBonus_Q5_40|GraveSpawnWeightBonus_Q6_40</t>
         </is>
@@ -1631,7 +1633,7 @@
         </is>
       </c>
       <c r="E13" t="inlineStr"/>
-      <c r="F13" s="6" t="n">
+      <c r="F13" s="5" t="n">
         <v>5</v>
       </c>
       <c r="G13" t="inlineStr">
@@ -1639,7 +1641,7 @@
           <t>Dig</t>
         </is>
       </c>
-      <c r="H13" s="3" t="inlineStr">
+      <c r="H13" t="inlineStr">
         <is>
           <t>GraveSpawnWeightBonus_Q4_50|GraveSpawnWeightBonus_Q5_50|GraveSpawnWeightBonus_Q6_50</t>
         </is>
@@ -1676,7 +1678,7 @@
           <t>1</t>
         </is>
       </c>
-      <c r="F14" s="6" t="inlineStr">
+      <c r="F14" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -1686,7 +1688,7 @@
           <t>Dig</t>
         </is>
       </c>
-      <c r="H14" s="4" t="inlineStr">
+      <c r="H14" s="7" t="inlineStr">
         <is>
           <t>DigOnGraveClear_1|ExplosiveThrowRadius_3|ExplosiveBlastRadius_1.5|ExplosiveBlastDamage_13|ExplosiveFlightSec_0.5|ExplosiveFuseSec_0.8|ExplosiveRingSec_0.5</t>
         </is>
@@ -1723,7 +1725,7 @@
           <t>1</t>
         </is>
       </c>
-      <c r="F15" s="6" t="n">
+      <c r="F15" s="5" t="n">
         <v>2</v>
       </c>
       <c r="G15" t="inlineStr">
@@ -1731,7 +1733,7 @@
           <t>Dig</t>
         </is>
       </c>
-      <c r="H15" s="4" t="inlineStr">
+      <c r="H15" s="7" t="inlineStr">
         <is>
           <t>DigOnGraveClear_1|ExplosiveThrowRadius_3|ExplosiveBlastRadius_1.5|ExplosiveBlastDamage_18|ExplosiveFlightSec_0.5|ExplosiveFuseSec_0.8|ExplosiveRingSec_0.5</t>
         </is>
@@ -1768,7 +1770,7 @@
           <t>1</t>
         </is>
       </c>
-      <c r="F16" s="6" t="n">
+      <c r="F16" s="5" t="n">
         <v>3</v>
       </c>
       <c r="G16" t="inlineStr">
@@ -1776,7 +1778,7 @@
           <t>Dig</t>
         </is>
       </c>
-      <c r="H16" s="4" t="inlineStr">
+      <c r="H16" s="7" t="inlineStr">
         <is>
           <t>DigOnGraveClear_1|ExplosiveThrowRadius_3|ExplosiveBlastRadius_1.5|ExplosiveBlastDamage_23|ExplosiveFlightSec_0.5|ExplosiveFuseSec_0.8|ExplosiveRingSec_0.5</t>
         </is>
@@ -1813,7 +1815,7 @@
           <t>1</t>
         </is>
       </c>
-      <c r="F17" s="6" t="n">
+      <c r="F17" s="5" t="n">
         <v>4</v>
       </c>
       <c r="G17" t="inlineStr">
@@ -1821,7 +1823,7 @@
           <t>Dig</t>
         </is>
       </c>
-      <c r="H17" s="4" t="inlineStr">
+      <c r="H17" s="7" t="inlineStr">
         <is>
           <t>DigOnGraveClear_1|ExplosiveThrowRadius_3|ExplosiveBlastRadius_1.5|ExplosiveBlastDamage_28|ExplosiveFlightSec_0.5|ExplosiveFuseSec_0.8|ExplosiveRingSec_0.5</t>
         </is>
@@ -1853,7 +1855,7 @@
           <t>Icon_Explosives</t>
         </is>
       </c>
-      <c r="F18" s="6" t="n">
+      <c r="F18" s="5" t="n">
         <v>5</v>
       </c>
       <c r="G18" t="inlineStr">
@@ -1861,7 +1863,7 @@
           <t>Dig</t>
         </is>
       </c>
-      <c r="H18" s="4" t="inlineStr">
+      <c r="H18" s="7" t="inlineStr">
         <is>
           <t>DigOnGraveClear_1|ExplosiveThrowRadius_3|ExplosiveBlastRadius_1.5|ExplosiveBlastDamage_33|ExplosiveFlightSec_0.5|ExplosiveFuseSec_0.8|ExplosiveRingSec_0.5</t>
         </is>
@@ -1898,7 +1900,7 @@
           <t>1</t>
         </is>
       </c>
-      <c r="F19" s="6" t="inlineStr">
+      <c r="F19" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -1908,7 +1910,7 @@
           <t>Dig</t>
         </is>
       </c>
-      <c r="H19" s="4" t="inlineStr">
+      <c r="H19" s="7" t="inlineStr">
         <is>
           <t>DigLightningIntervalSec_15|DigLightningFrameSec_0.05|DigLightningPreviewSec_2</t>
         </is>
@@ -1945,7 +1947,7 @@
           <t>1</t>
         </is>
       </c>
-      <c r="F20" s="6" t="n">
+      <c r="F20" s="5" t="n">
         <v>2</v>
       </c>
       <c r="G20" t="inlineStr">
@@ -1953,7 +1955,7 @@
           <t>Dig</t>
         </is>
       </c>
-      <c r="H20" s="4" t="inlineStr">
+      <c r="H20" s="7" t="inlineStr">
         <is>
           <t>DigLightningIntervalSec_13|DigLightningFrameSec_0.05|DigLightningPreviewSec_2</t>
         </is>
@@ -1990,7 +1992,7 @@
           <t>1</t>
         </is>
       </c>
-      <c r="F21" s="6" t="n">
+      <c r="F21" s="5" t="n">
         <v>3</v>
       </c>
       <c r="G21" t="inlineStr">
@@ -1998,7 +2000,7 @@
           <t>Dig</t>
         </is>
       </c>
-      <c r="H21" s="4" t="inlineStr">
+      <c r="H21" s="7" t="inlineStr">
         <is>
           <t>DigLightningIntervalSec_11|DigLightningFrameSec_0.05|DigLightningPreviewSec_2</t>
         </is>
@@ -2035,7 +2037,7 @@
           <t>1</t>
         </is>
       </c>
-      <c r="F22" s="6" t="n">
+      <c r="F22" s="5" t="n">
         <v>4</v>
       </c>
       <c r="G22" t="inlineStr">
@@ -2043,7 +2045,7 @@
           <t>Dig</t>
         </is>
       </c>
-      <c r="H22" s="4" t="inlineStr">
+      <c r="H22" s="7" t="inlineStr">
         <is>
           <t>DigLightningIntervalSec_9|DigLightningFrameSec_0.05|DigLightningPreviewSec_2</t>
         </is>
@@ -2075,7 +2077,7 @@
           <t>Icon_Elctr</t>
         </is>
       </c>
-      <c r="F23" s="6" t="n">
+      <c r="F23" s="5" t="n">
         <v>5</v>
       </c>
       <c r="G23" t="inlineStr">
@@ -2083,7 +2085,7 @@
           <t>Dig</t>
         </is>
       </c>
-      <c r="H23" s="4" t="inlineStr">
+      <c r="H23" s="7" t="inlineStr">
         <is>
           <t>DigLightningIntervalSec_7|DigLightningFrameSec_0.05|DigLightningPreviewSec_2</t>
         </is>
@@ -2120,7 +2122,7 @@
           <t>1</t>
         </is>
       </c>
-      <c r="F24" s="6" t="inlineStr">
+      <c r="F24" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -2137,7 +2139,7 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>每级增加过程生成坟墓数量+1（1级）</t>
+          <t>每级增加挖坟过程生成坟墓数量+1（1级）</t>
         </is>
       </c>
     </row>
@@ -2167,7 +2169,7 @@
           <t>1</t>
         </is>
       </c>
-      <c r="F25" s="6" t="n">
+      <c r="F25" s="5" t="n">
         <v>2</v>
       </c>
       <c r="G25" t="inlineStr">
@@ -2182,7 +2184,7 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>每级增加过程生成坟墓数量+1（2级）</t>
+          <t>每级增加挖坟过程生成坟墓数量+1（2级）</t>
         </is>
       </c>
     </row>
@@ -2212,7 +2214,7 @@
           <t>1</t>
         </is>
       </c>
-      <c r="F26" s="6" t="n">
+      <c r="F26" s="5" t="n">
         <v>3</v>
       </c>
       <c r="G26" t="inlineStr">
@@ -2227,7 +2229,7 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>每级增加过程生成坟墓数量+1（3级）</t>
+          <t>每级增加挖坟过程生成坟墓数量+1（3级）</t>
         </is>
       </c>
     </row>
@@ -2257,7 +2259,7 @@
           <t>1</t>
         </is>
       </c>
-      <c r="F27" s="6" t="n">
+      <c r="F27" s="5" t="n">
         <v>4</v>
       </c>
       <c r="G27" t="inlineStr">
@@ -2272,7 +2274,7 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>每级增加过程生成坟墓数量+1（4级）</t>
+          <t>每级增加挖坟过程生成坟墓数量+1（4级）</t>
         </is>
       </c>
     </row>
@@ -2297,7 +2299,7 @@
           <t>Icon_Detector</t>
         </is>
       </c>
-      <c r="F28" s="6" t="n">
+      <c r="F28" s="5" t="n">
         <v>5</v>
       </c>
       <c r="G28" t="inlineStr">
@@ -2312,24 +2314,684 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>每级增加过程生成坟墓数量+1（满级）</t>
+          <t>每级增加挖坟过程生成坟墓数量+1（满级）</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="F29" s="6" t="n"/>
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Equip_HumanToken</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>人类信物</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Icon_HumanToken</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F29" s="5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Dig</t>
+        </is>
+      </c>
+      <c r="H29" s="6" t="inlineStr">
+        <is>
+          <t>GraveSpawnWeightBonus_Q16_10|GraveSpawnWeightBonus_Q17_10|GraveSpawnWeightBonus_Q18_10|GraveSpawnWeightBonus_Q19_10</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>增加发现人类坟墓的概率</t>
+        </is>
+      </c>
     </row>
     <row r="30">
-      <c r="F30" s="6" t="n"/>
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Equip_HumanToken</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>人类信物</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Icon_HumanToken</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F30" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Dig</t>
+        </is>
+      </c>
+      <c r="H30" s="6" t="inlineStr">
+        <is>
+          <t>GraveSpawnWeightBonus_Q16_15|GraveSpawnWeightBonus_Q17_15|GraveSpawnWeightBonus_Q18_15|GraveSpawnWeightBonus_Q19_15</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>增加发现人类坟墓的概率</t>
+        </is>
+      </c>
     </row>
     <row r="31">
-      <c r="F31" s="6" t="n"/>
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Equip_HumanToken</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>人类信物</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Icon_HumanToken</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F31" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Dig</t>
+        </is>
+      </c>
+      <c r="H31" s="6" t="inlineStr">
+        <is>
+          <t>GraveSpawnWeightBonus_Q16_20|GraveSpawnWeightBonus_Q17_20|GraveSpawnWeightBonus_Q18_20|GraveSpawnWeightBonus_Q19_20</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>增加发现人类坟墓的概率</t>
+        </is>
+      </c>
     </row>
     <row r="32">
-      <c r="F32" s="6" t="n"/>
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Equip_HumanToken</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>人类信物</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Icon_HumanToken</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F32" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Dig</t>
+        </is>
+      </c>
+      <c r="H32" s="6" t="inlineStr">
+        <is>
+          <t>GraveSpawnWeightBonus_Q16_25|GraveSpawnWeightBonus_Q17_25|GraveSpawnWeightBonus_Q18_25|GraveSpawnWeightBonus_Q19_25</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>增加发现人类坟墓的概率</t>
+        </is>
+      </c>
     </row>
     <row r="33">
-      <c r="F33" s="6" t="n"/>
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Equip_HumanToken</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>人类信物</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Icon_HumanToken</t>
+        </is>
+      </c>
+      <c r="F33" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Dig</t>
+        </is>
+      </c>
+      <c r="H33" s="6" t="inlineStr">
+        <is>
+          <t>GraveSpawnWeightBonus_Q16_30|GraveSpawnWeightBonus_Q17_30|GraveSpawnWeightBonus_Q18_30|GraveSpawnWeightBonus_Q19_30</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>增加发现人类坟墓的概率</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Equip_ElfToken</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>精灵信物</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Icon_ElfToken</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F34" s="5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Dig</t>
+        </is>
+      </c>
+      <c r="H34" s="6" t="inlineStr">
+        <is>
+          <t>GraveSpawnWeightBonus_Q20_10|GraveSpawnWeightBonus_Q21_10|GraveSpawnWeightBonus_Q22_10|GraveSpawnWeightBonus_Q23_10</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>增加发现精灵族坟墓的概率</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Equip_ElfToken</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>精灵信物</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Icon_ElfToken</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F35" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Dig</t>
+        </is>
+      </c>
+      <c r="H35" s="6" t="inlineStr">
+        <is>
+          <t>GraveSpawnWeightBonus_Q20_15|GraveSpawnWeightBonus_Q21_15|GraveSpawnWeightBonus_Q22_15|GraveSpawnWeightBonus_Q23_15</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>增加发现精灵族坟墓的概率</t>
+        </is>
+      </c>
+      <c r="J35" s="7" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Equip_ElfToken</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>精灵信物</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Icon_ElfToken</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F36" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Dig</t>
+        </is>
+      </c>
+      <c r="H36" s="6" t="inlineStr">
+        <is>
+          <t>GraveSpawnWeightBonus_Q20_20|GraveSpawnWeightBonus_Q21_20|GraveSpawnWeightBonus_Q22_20|GraveSpawnWeightBonus_Q23_20</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>增加发现精灵族坟墓的概率</t>
+        </is>
+      </c>
+      <c r="J36" s="7" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Equip_ElfToken</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>精灵信物</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Icon_ElfToken</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F37" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Dig</t>
+        </is>
+      </c>
+      <c r="H37" s="6" t="inlineStr">
+        <is>
+          <t>GraveSpawnWeightBonus_Q20_25|GraveSpawnWeightBonus_Q21_25|GraveSpawnWeightBonus_Q22_25|GraveSpawnWeightBonus_Q23_25</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>增加发现精灵族坟墓的概率</t>
+        </is>
+      </c>
+      <c r="J37" s="7" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Equip_ElfToken</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>精灵信物</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Icon_ElfToken</t>
+        </is>
+      </c>
+      <c r="F38" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Dig</t>
+        </is>
+      </c>
+      <c r="H38" s="6" t="inlineStr">
+        <is>
+          <t>GraveSpawnWeightBonus_Q20_30|GraveSpawnWeightBonus_Q21_30|GraveSpawnWeightBonus_Q22_30|GraveSpawnWeightBonus_Q23_30</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>增加发现精灵族坟墓的概率</t>
+        </is>
+      </c>
+      <c r="J38" s="7" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Equip_OrcToken</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C39" s="7" t="inlineStr">
+        <is>
+          <t>兽人信物</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Icon_OrcToken</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F39" s="5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Dig</t>
+        </is>
+      </c>
+      <c r="H39" s="6" t="inlineStr">
+        <is>
+          <t>GraveSpawnWeightBonus_Q24_10|GraveSpawnWeightBonus_Q25_10|GraveSpawnWeightBonus_Q26_10|GraveSpawnWeightBonus_Q27_10</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>增加发现兽人坟墓的概率</t>
+        </is>
+      </c>
+      <c r="J39" s="7" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Equip_OrcToken</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C40" s="7" t="inlineStr">
+        <is>
+          <t>兽人信物</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Icon_OrcToken</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F40" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Dig</t>
+        </is>
+      </c>
+      <c r="H40" s="6" t="inlineStr">
+        <is>
+          <t>GraveSpawnWeightBonus_Q24_15|GraveSpawnWeightBonus_Q25_15|GraveSpawnWeightBonus_Q26_15|GraveSpawnWeightBonus_Q27_15</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>增加发现兽人坟墓的概率</t>
+        </is>
+      </c>
+      <c r="J40" s="7" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Equip_OrcToken</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C41" s="7" t="inlineStr">
+        <is>
+          <t>兽人信物</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Icon_OrcToken</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F41" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Dig</t>
+        </is>
+      </c>
+      <c r="H41" s="6" t="inlineStr">
+        <is>
+          <t>GraveSpawnWeightBonus_Q24_20|GraveSpawnWeightBonus_Q25_20|GraveSpawnWeightBonus_Q26_20|GraveSpawnWeightBonus_Q27_20</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>增加发现兽人坟墓的概率</t>
+        </is>
+      </c>
+      <c r="J41" s="7" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Equip_OrcToken</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C42" s="7" t="inlineStr">
+        <is>
+          <t>兽人信物</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Icon_OrcToken</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F42" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Dig</t>
+        </is>
+      </c>
+      <c r="H42" s="6" t="inlineStr">
+        <is>
+          <t>GraveSpawnWeightBonus_Q24_25|GraveSpawnWeightBonus_Q25_25|GraveSpawnWeightBonus_Q26_25|GraveSpawnWeightBonus_Q27_25</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>增加发现兽人坟墓的概率</t>
+        </is>
+      </c>
+      <c r="J42" s="7" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Equip_OrcToken</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C43" s="7" t="inlineStr">
+        <is>
+          <t>兽人信物</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Icon_OrcToken</t>
+        </is>
+      </c>
+      <c r="F43" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Dig</t>
+        </is>
+      </c>
+      <c r="H43" s="6" t="inlineStr">
+        <is>
+          <t>GraveSpawnWeightBonus_Q24_30|GraveSpawnWeightBonus_Q25_30|GraveSpawnWeightBonus_Q26_30|GraveSpawnWeightBonus_Q27_30</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>增加发现兽人坟墓的概率</t>
+        </is>
+      </c>
+      <c r="J43" s="7" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>